<commit_message>
Fencing pay-and-charge workbook to the cent: $255,218.20 / $364,816.40
Rebuilt from read-only dumps of the live page: the charge column is the
page's own lines on Advanced's quantities, so the total ties to the
P&L's V8 fencing charge to the cent; the pay side carries the receipted
order once.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Fencing_We_Pay_We_Charge_25Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Fencing_We_Pay_We_Charge_25Oct2026.xlsx
@@ -503,7 +503,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AUD ex GST · 25 Oct 2026</t>
+          <t>AUD ex GST · 25 Oct 2026 · the same quantity both sides; the totals are the page's own, to the cent</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
         <v>16.1607</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>146020</v>
+        <v>146019.97</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         <v>25.53</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>94014.23</v>
+        <v>94014.35000000001</v>
       </c>
     </row>
     <row r="7">
@@ -649,7 +649,7 @@
         <v>7.51</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>16484.45</v>
+        <v>16484.48</v>
       </c>
     </row>
     <row r="9">
@@ -676,7 +676,7 @@
         <v>9.6511</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>2200.45</v>
+        <v>2200.46</v>
       </c>
     </row>
     <row r="10">
@@ -757,7 +757,7 @@
         <v>36.1839</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>796.05</v>
+        <v>796.04</v>
       </c>
     </row>
     <row r="13">
@@ -978,7 +978,7 @@
       </c>
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="8" t="n">
-        <v>364816.28</v>
+        <v>364816.4</v>
       </c>
     </row>
     <row r="22">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="G22" s="8" t="n">
-        <v>109598.08</v>
+        <v>109598.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>